<commit_message>
Day 19 JSON and POM format data driven
</commit_message>
<xml_diff>
--- a/playwright/testData/textData.xlsx
+++ b/playwright/testData/textData.xlsx
@@ -4,17 +4,55 @@
   <fileVersion rupBuild="9303" lowestEdited="5" lastEdited="5" appName="xl"/>
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="0"/>
+    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet r:id="rId1" sheetId="1" name="Sheet 1"/>
+    <sheet r:id="rId2" sheetId="2" name="Sheet 2"/>
+    <sheet r:id="rId3" sheetId="3" name="Sheet 3"/>
   </sheets>
   <calcPr fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="24">
+  <si>
+    <t>shoes for man stylish</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>shoes for woman</t>
+  </si>
+  <si>
+    <t>shoes for men sports</t>
+  </si>
+  <si>
+    <t>shoes for men casual</t>
+  </si>
+  <si>
+    <t>shoes rack with door</t>
+  </si>
+  <si>
+    <t>shoes for men formal</t>
+  </si>
+  <si>
+    <t>shoes for man stylish nike</t>
+  </si>
+  <si>
+    <t>shoes for men campus sports</t>
+  </si>
+  <si>
+    <t>shoes cleaner</t>
+  </si>
+  <si>
+    <t>shoes for men adidas stylish</t>
+  </si>
+  <si>
+    <t>newShee2</t>
+  </si>
   <si>
     <t>Username</t>
   </si>
@@ -57,13 +95,19 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
   <numFmts count="0"/>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
@@ -79,7 +123,7 @@
     </font>
     <font>
       <sz val="11"/>
-      <color theme="1"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -97,7 +141,14 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="13">
+  <borders count="14">
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
     <border>
       <left/>
       <right/>
@@ -289,18 +340,33 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="21">
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="general" wrapText="1"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" quotePrefix="1" applyAlignment="1">
+      <alignment horizontal="general"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="general"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="general" wrapText="1"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="general"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="3" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="3" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="4" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
@@ -309,29 +375,32 @@
     <xf xfId="0" numFmtId="0" borderId="5" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="6" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="6" applyBorder="1" fontId="4" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="7" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="7" applyBorder="1" fontId="4" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="8" applyBorder="1" fontId="3" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="8" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="9" applyBorder="1" fontId="3" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="9" applyBorder="1" fontId="4" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="10" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="10" applyBorder="1" fontId="4" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="11" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="12" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="12" applyBorder="1" fontId="4" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
+    <xf xfId="0" numFmtId="0" borderId="13" applyBorder="1" fontId="4" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general" wrapText="1"/>
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -638,54 +707,791 @@
   <dimension ref="A1:C4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="14" width="26.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="14" width="16.290714285714284" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="14" width="16.290714285714284" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="20" width="26.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="20" width="16.290714285714284" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="20" width="16.290714285714284" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="20.55" customFormat="1" s="1">
-      <c r="A1" s="2" t="s">
+    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="20.55" customFormat="1" s="4">
+      <c r="A1" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="B1" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1" s="10" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="17.25" customFormat="1" s="4">
+      <c r="A2" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="B2" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="C2" s="13" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="17.25" customFormat="1" s="4">
+      <c r="A3" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="B3" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="C3" s="16" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18" customFormat="1" s="4">
+      <c r="A4" s="17" t="s">
+        <v>21</v>
+      </c>
+      <c r="B4" s="18" t="s">
+        <v>22</v>
+      </c>
+      <c r="C4" s="19" t="s">
+        <v>23</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <sheetPr>
+    <outlinePr summaryBelow="0"/>
+  </sheetPr>
+  <dimension ref="A1:A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" style="7" width="12.43357142857143" customWidth="1" bestFit="1"/>
+  </cols>
+  <sheetData>
+    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="17.25" customFormat="1" s="4">
+      <c r="A1" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <sheetPr>
+    <outlinePr summaryBelow="0"/>
+  </sheetPr>
+  <dimension ref="A1:AY10"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" style="6" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="7" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="7" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="7" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="7" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="7" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="7" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="8" max="8" style="7" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="9" max="9" style="7" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="10" max="10" style="7" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="11" max="11" style="7" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="12" max="12" style="7" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="13" max="13" style="7" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="14" max="14" style="7" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="15" max="15" style="7" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="16" max="16" style="7" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="17" max="17" style="7" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="18" max="18" style="7" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="19" max="19" style="7" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="20" max="20" style="7" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="21" max="21" style="7" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="22" max="22" style="7" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="23" max="23" style="7" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="24" max="24" style="7" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="25" max="25" style="7" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="26" max="26" style="7" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="27" max="27" style="7" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="28" max="28" style="7" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="29" max="29" style="7" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="30" max="30" style="7" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="31" max="31" style="7" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="32" max="32" style="7" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="33" max="33" style="7" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="34" max="34" style="7" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="35" max="35" style="7" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="36" max="36" style="7" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="37" max="37" style="7" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="38" max="38" style="7" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="39" max="39" style="7" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="40" max="40" style="7" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="41" max="41" style="7" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="42" max="42" style="7" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="43" max="43" style="7" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="44" max="44" style="7" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="45" max="45" style="7" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="46" max="46" style="7" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="47" max="47" style="7" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="48" max="48" style="7" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="49" max="49" style="7" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="50" max="50" style="7" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="51" max="51" style="7" width="12.43357142857143" customWidth="1" bestFit="1"/>
+  </cols>
+  <sheetData>
+    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="29.25">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="4" t="s">
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="L1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="M1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="N1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="O1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="P1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="Q1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="R1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="S1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="T1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="U1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="V1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="W1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="X1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="Y1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="Z1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="AA1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="AB1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="AC1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="AD1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="AE1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="AF1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="AG1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="AH1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="AI1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="AJ1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="AK1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="AL1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="AM1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="AN1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="AO1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="AP1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="AQ1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="AR1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="AS1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="AT1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="AU1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="AV1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="AW1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="AX1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="AY1" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="29.25">
+      <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
+      <c r="G2" s="3"/>
+      <c r="H2" s="3"/>
+      <c r="I2" s="3"/>
+      <c r="J2" s="3"/>
+      <c r="K2" s="3"/>
+      <c r="L2" s="3"/>
+      <c r="M2" s="3"/>
+      <c r="N2" s="3"/>
+      <c r="O2" s="3"/>
+      <c r="P2" s="3"/>
+      <c r="Q2" s="3"/>
+      <c r="R2" s="3"/>
+      <c r="S2" s="3"/>
+      <c r="T2" s="3"/>
+      <c r="U2" s="3"/>
+      <c r="V2" s="3"/>
+      <c r="W2" s="3"/>
+      <c r="X2" s="3"/>
+      <c r="Y2" s="3"/>
+      <c r="Z2" s="3"/>
+      <c r="AA2" s="3"/>
+      <c r="AB2" s="3"/>
+      <c r="AC2" s="3"/>
+      <c r="AD2" s="3"/>
+      <c r="AE2" s="3"/>
+      <c r="AF2" s="3"/>
+      <c r="AG2" s="3"/>
+      <c r="AH2" s="3"/>
+      <c r="AI2" s="3"/>
+      <c r="AJ2" s="3"/>
+      <c r="AK2" s="3"/>
+      <c r="AL2" s="3"/>
+      <c r="AM2" s="3"/>
+      <c r="AN2" s="3"/>
+      <c r="AO2" s="3"/>
+      <c r="AP2" s="3"/>
+      <c r="AQ2" s="3"/>
+      <c r="AR2" s="3"/>
+      <c r="AS2" s="3"/>
+      <c r="AT2" s="3"/>
+      <c r="AU2" s="3"/>
+      <c r="AV2" s="3"/>
+      <c r="AW2" s="3"/>
+      <c r="AX2" s="3"/>
+      <c r="AY2" s="3"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="17.25" customFormat="1" s="1">
-      <c r="A2" s="5" t="s">
+    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="29.25">
+      <c r="A3" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="6" t="s">
+      <c r="B3" s="3"/>
+      <c r="C3" s="3"/>
+      <c r="D3" s="3"/>
+      <c r="E3" s="3"/>
+      <c r="F3" s="3"/>
+      <c r="G3" s="3"/>
+      <c r="H3" s="3"/>
+      <c r="I3" s="3"/>
+      <c r="J3" s="3"/>
+      <c r="K3" s="3"/>
+      <c r="L3" s="3"/>
+      <c r="M3" s="3"/>
+      <c r="N3" s="3"/>
+      <c r="O3" s="3"/>
+      <c r="P3" s="3"/>
+      <c r="Q3" s="3"/>
+      <c r="R3" s="3"/>
+      <c r="S3" s="3"/>
+      <c r="T3" s="3"/>
+      <c r="U3" s="3"/>
+      <c r="V3" s="3"/>
+      <c r="W3" s="3"/>
+      <c r="X3" s="3"/>
+      <c r="Y3" s="3"/>
+      <c r="Z3" s="3"/>
+      <c r="AA3" s="3"/>
+      <c r="AB3" s="3"/>
+      <c r="AC3" s="3"/>
+      <c r="AD3" s="3"/>
+      <c r="AE3" s="3"/>
+      <c r="AF3" s="3"/>
+      <c r="AG3" s="3"/>
+      <c r="AH3" s="3"/>
+      <c r="AI3" s="3"/>
+      <c r="AJ3" s="3"/>
+      <c r="AK3" s="3"/>
+      <c r="AL3" s="3"/>
+      <c r="AM3" s="3"/>
+      <c r="AN3" s="3"/>
+      <c r="AO3" s="3"/>
+      <c r="AP3" s="3"/>
+      <c r="AQ3" s="3"/>
+      <c r="AR3" s="3"/>
+      <c r="AS3" s="3"/>
+      <c r="AT3" s="3"/>
+      <c r="AU3" s="3"/>
+      <c r="AV3" s="3"/>
+      <c r="AW3" s="3"/>
+      <c r="AX3" s="3"/>
+      <c r="AY3" s="3"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="29.25">
+      <c r="A4" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="7" t="s">
+      <c r="B4" s="3"/>
+      <c r="C4" s="3"/>
+      <c r="D4" s="3"/>
+      <c r="E4" s="3"/>
+      <c r="F4" s="3"/>
+      <c r="G4" s="3"/>
+      <c r="H4" s="3"/>
+      <c r="I4" s="3"/>
+      <c r="J4" s="3"/>
+      <c r="K4" s="3"/>
+      <c r="L4" s="3"/>
+      <c r="M4" s="3"/>
+      <c r="N4" s="3"/>
+      <c r="O4" s="3"/>
+      <c r="P4" s="3"/>
+      <c r="Q4" s="3"/>
+      <c r="R4" s="3"/>
+      <c r="S4" s="3"/>
+      <c r="T4" s="3"/>
+      <c r="U4" s="3"/>
+      <c r="V4" s="3"/>
+      <c r="W4" s="3"/>
+      <c r="X4" s="3"/>
+      <c r="Y4" s="3"/>
+      <c r="Z4" s="3"/>
+      <c r="AA4" s="3"/>
+      <c r="AB4" s="3"/>
+      <c r="AC4" s="3"/>
+      <c r="AD4" s="3"/>
+      <c r="AE4" s="3"/>
+      <c r="AF4" s="3"/>
+      <c r="AG4" s="3"/>
+      <c r="AH4" s="3"/>
+      <c r="AI4" s="3"/>
+      <c r="AJ4" s="3"/>
+      <c r="AK4" s="3"/>
+      <c r="AL4" s="3"/>
+      <c r="AM4" s="3"/>
+      <c r="AN4" s="3"/>
+      <c r="AO4" s="3"/>
+      <c r="AP4" s="3"/>
+      <c r="AQ4" s="3"/>
+      <c r="AR4" s="3"/>
+      <c r="AS4" s="3"/>
+      <c r="AT4" s="3"/>
+      <c r="AU4" s="3"/>
+      <c r="AV4" s="3"/>
+      <c r="AW4" s="3"/>
+      <c r="AX4" s="3"/>
+      <c r="AY4" s="3"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="29.25">
+      <c r="A5" s="1" t="s">
         <v>5</v>
       </c>
+      <c r="B5" s="3"/>
+      <c r="C5" s="3"/>
+      <c r="D5" s="3"/>
+      <c r="E5" s="3"/>
+      <c r="F5" s="3"/>
+      <c r="G5" s="3"/>
+      <c r="H5" s="3"/>
+      <c r="I5" s="3"/>
+      <c r="J5" s="3"/>
+      <c r="K5" s="3"/>
+      <c r="L5" s="3"/>
+      <c r="M5" s="3"/>
+      <c r="N5" s="3"/>
+      <c r="O5" s="3"/>
+      <c r="P5" s="3"/>
+      <c r="Q5" s="3"/>
+      <c r="R5" s="3"/>
+      <c r="S5" s="3"/>
+      <c r="T5" s="3"/>
+      <c r="U5" s="3"/>
+      <c r="V5" s="3"/>
+      <c r="W5" s="3"/>
+      <c r="X5" s="3"/>
+      <c r="Y5" s="3"/>
+      <c r="Z5" s="3"/>
+      <c r="AA5" s="3"/>
+      <c r="AB5" s="3"/>
+      <c r="AC5" s="3"/>
+      <c r="AD5" s="3"/>
+      <c r="AE5" s="3"/>
+      <c r="AF5" s="3"/>
+      <c r="AG5" s="3"/>
+      <c r="AH5" s="3"/>
+      <c r="AI5" s="3"/>
+      <c r="AJ5" s="3"/>
+      <c r="AK5" s="3"/>
+      <c r="AL5" s="3"/>
+      <c r="AM5" s="3"/>
+      <c r="AN5" s="3"/>
+      <c r="AO5" s="3"/>
+      <c r="AP5" s="3"/>
+      <c r="AQ5" s="3"/>
+      <c r="AR5" s="3"/>
+      <c r="AS5" s="3"/>
+      <c r="AT5" s="3"/>
+      <c r="AU5" s="3"/>
+      <c r="AV5" s="3"/>
+      <c r="AW5" s="3"/>
+      <c r="AX5" s="3"/>
+      <c r="AY5" s="3"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="17.25" customFormat="1" s="1">
-      <c r="A3" s="8" t="s">
+    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="29.25">
+      <c r="A6" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="9" t="s">
+      <c r="B6" s="3"/>
+      <c r="C6" s="3"/>
+      <c r="D6" s="3"/>
+      <c r="E6" s="3"/>
+      <c r="F6" s="3"/>
+      <c r="G6" s="3"/>
+      <c r="H6" s="3"/>
+      <c r="I6" s="3"/>
+      <c r="J6" s="3"/>
+      <c r="K6" s="3"/>
+      <c r="L6" s="3"/>
+      <c r="M6" s="3"/>
+      <c r="N6" s="3"/>
+      <c r="O6" s="3"/>
+      <c r="P6" s="3"/>
+      <c r="Q6" s="3"/>
+      <c r="R6" s="3"/>
+      <c r="S6" s="3"/>
+      <c r="T6" s="3"/>
+      <c r="U6" s="3"/>
+      <c r="V6" s="3"/>
+      <c r="W6" s="3"/>
+      <c r="X6" s="3"/>
+      <c r="Y6" s="3"/>
+      <c r="Z6" s="3"/>
+      <c r="AA6" s="3"/>
+      <c r="AB6" s="3"/>
+      <c r="AC6" s="3"/>
+      <c r="AD6" s="3"/>
+      <c r="AE6" s="3"/>
+      <c r="AF6" s="3"/>
+      <c r="AG6" s="3"/>
+      <c r="AH6" s="3"/>
+      <c r="AI6" s="3"/>
+      <c r="AJ6" s="3"/>
+      <c r="AK6" s="3"/>
+      <c r="AL6" s="3"/>
+      <c r="AM6" s="3"/>
+      <c r="AN6" s="3"/>
+      <c r="AO6" s="3"/>
+      <c r="AP6" s="3"/>
+      <c r="AQ6" s="3"/>
+      <c r="AR6" s="3"/>
+      <c r="AS6" s="3"/>
+      <c r="AT6" s="3"/>
+      <c r="AU6" s="3"/>
+      <c r="AV6" s="3"/>
+      <c r="AW6" s="3"/>
+      <c r="AX6" s="3"/>
+      <c r="AY6" s="3"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="40.5">
+      <c r="A7" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C3" s="10" t="s">
+      <c r="B7" s="3"/>
+      <c r="C7" s="3"/>
+      <c r="D7" s="3"/>
+      <c r="E7" s="3"/>
+      <c r="F7" s="3"/>
+      <c r="G7" s="3"/>
+      <c r="H7" s="3"/>
+      <c r="I7" s="3"/>
+      <c r="J7" s="3"/>
+      <c r="K7" s="3"/>
+      <c r="L7" s="3"/>
+      <c r="M7" s="3"/>
+      <c r="N7" s="3"/>
+      <c r="O7" s="3"/>
+      <c r="P7" s="3"/>
+      <c r="Q7" s="3"/>
+      <c r="R7" s="3"/>
+      <c r="S7" s="3"/>
+      <c r="T7" s="3"/>
+      <c r="U7" s="3"/>
+      <c r="V7" s="3"/>
+      <c r="W7" s="3"/>
+      <c r="X7" s="3"/>
+      <c r="Y7" s="3"/>
+      <c r="Z7" s="3"/>
+      <c r="AA7" s="3"/>
+      <c r="AB7" s="3"/>
+      <c r="AC7" s="3"/>
+      <c r="AD7" s="3"/>
+      <c r="AE7" s="3"/>
+      <c r="AF7" s="3"/>
+      <c r="AG7" s="3"/>
+      <c r="AH7" s="3"/>
+      <c r="AI7" s="3"/>
+      <c r="AJ7" s="3"/>
+      <c r="AK7" s="3"/>
+      <c r="AL7" s="3"/>
+      <c r="AM7" s="3"/>
+      <c r="AN7" s="3"/>
+      <c r="AO7" s="3"/>
+      <c r="AP7" s="3"/>
+      <c r="AQ7" s="3"/>
+      <c r="AR7" s="3"/>
+      <c r="AS7" s="3"/>
+      <c r="AT7" s="3"/>
+      <c r="AU7" s="3"/>
+      <c r="AV7" s="3"/>
+      <c r="AW7" s="3"/>
+      <c r="AX7" s="3"/>
+      <c r="AY7" s="3"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="40.5">
+      <c r="A8" s="1" t="s">
         <v>8</v>
       </c>
+      <c r="B8" s="3"/>
+      <c r="C8" s="3"/>
+      <c r="D8" s="3"/>
+      <c r="E8" s="3"/>
+      <c r="F8" s="3"/>
+      <c r="G8" s="3"/>
+      <c r="H8" s="3"/>
+      <c r="I8" s="3"/>
+      <c r="J8" s="3"/>
+      <c r="K8" s="3"/>
+      <c r="L8" s="3"/>
+      <c r="M8" s="3"/>
+      <c r="N8" s="3"/>
+      <c r="O8" s="3"/>
+      <c r="P8" s="3"/>
+      <c r="Q8" s="3"/>
+      <c r="R8" s="3"/>
+      <c r="S8" s="3"/>
+      <c r="T8" s="3"/>
+      <c r="U8" s="3"/>
+      <c r="V8" s="3"/>
+      <c r="W8" s="3"/>
+      <c r="X8" s="3"/>
+      <c r="Y8" s="3"/>
+      <c r="Z8" s="3"/>
+      <c r="AA8" s="3"/>
+      <c r="AB8" s="3"/>
+      <c r="AC8" s="3"/>
+      <c r="AD8" s="3"/>
+      <c r="AE8" s="3"/>
+      <c r="AF8" s="3"/>
+      <c r="AG8" s="3"/>
+      <c r="AH8" s="3"/>
+      <c r="AI8" s="3"/>
+      <c r="AJ8" s="3"/>
+      <c r="AK8" s="3"/>
+      <c r="AL8" s="3"/>
+      <c r="AM8" s="3"/>
+      <c r="AN8" s="3"/>
+      <c r="AO8" s="3"/>
+      <c r="AP8" s="3"/>
+      <c r="AQ8" s="3"/>
+      <c r="AR8" s="3"/>
+      <c r="AS8" s="3"/>
+      <c r="AT8" s="3"/>
+      <c r="AU8" s="3"/>
+      <c r="AV8" s="3"/>
+      <c r="AW8" s="3"/>
+      <c r="AX8" s="3"/>
+      <c r="AY8" s="3"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18" customFormat="1" s="1">
-      <c r="A4" s="11" t="s">
+    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="29.25">
+      <c r="A9" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="12" t="s">
+      <c r="B9" s="3"/>
+      <c r="C9" s="3"/>
+      <c r="D9" s="3"/>
+      <c r="E9" s="3"/>
+      <c r="F9" s="3"/>
+      <c r="G9" s="3"/>
+      <c r="H9" s="3"/>
+      <c r="I9" s="3"/>
+      <c r="J9" s="3"/>
+      <c r="K9" s="3"/>
+      <c r="L9" s="3"/>
+      <c r="M9" s="3"/>
+      <c r="N9" s="3"/>
+      <c r="O9" s="3"/>
+      <c r="P9" s="3"/>
+      <c r="Q9" s="3"/>
+      <c r="R9" s="3"/>
+      <c r="S9" s="3"/>
+      <c r="T9" s="3"/>
+      <c r="U9" s="3"/>
+      <c r="V9" s="3"/>
+      <c r="W9" s="3"/>
+      <c r="X9" s="3"/>
+      <c r="Y9" s="3"/>
+      <c r="Z9" s="3"/>
+      <c r="AA9" s="3"/>
+      <c r="AB9" s="3"/>
+      <c r="AC9" s="3"/>
+      <c r="AD9" s="3"/>
+      <c r="AE9" s="3"/>
+      <c r="AF9" s="3"/>
+      <c r="AG9" s="3"/>
+      <c r="AH9" s="3"/>
+      <c r="AI9" s="3"/>
+      <c r="AJ9" s="3"/>
+      <c r="AK9" s="3"/>
+      <c r="AL9" s="3"/>
+      <c r="AM9" s="3"/>
+      <c r="AN9" s="3"/>
+      <c r="AO9" s="3"/>
+      <c r="AP9" s="3"/>
+      <c r="AQ9" s="3"/>
+      <c r="AR9" s="3"/>
+      <c r="AS9" s="3"/>
+      <c r="AT9" s="3"/>
+      <c r="AU9" s="3"/>
+      <c r="AV9" s="3"/>
+      <c r="AW9" s="3"/>
+      <c r="AX9" s="3"/>
+      <c r="AY9" s="3"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="40.5" customFormat="1" s="4">
+      <c r="A10" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="C4" s="13" t="s">
-        <v>11</v>
-      </c>
+      <c r="B10" s="1"/>
+      <c r="C10" s="1"/>
+      <c r="D10" s="1"/>
+      <c r="E10" s="1"/>
+      <c r="F10" s="1"/>
+      <c r="G10" s="1"/>
+      <c r="H10" s="1"/>
+      <c r="I10" s="1"/>
+      <c r="J10" s="1"/>
+      <c r="K10" s="1"/>
+      <c r="L10" s="1"/>
+      <c r="M10" s="1"/>
+      <c r="N10" s="1"/>
+      <c r="O10" s="1"/>
+      <c r="P10" s="1"/>
+      <c r="Q10" s="1"/>
+      <c r="R10" s="1"/>
+      <c r="S10" s="1"/>
+      <c r="T10" s="1"/>
+      <c r="U10" s="1"/>
+      <c r="V10" s="1"/>
+      <c r="W10" s="1"/>
+      <c r="X10" s="1"/>
+      <c r="Y10" s="1"/>
+      <c r="Z10" s="1"/>
+      <c r="AA10" s="1"/>
+      <c r="AB10" s="1"/>
+      <c r="AC10" s="1"/>
+      <c r="AD10" s="1"/>
+      <c r="AE10" s="1"/>
+      <c r="AF10" s="1"/>
+      <c r="AG10" s="1"/>
+      <c r="AH10" s="1"/>
+      <c r="AI10" s="1"/>
+      <c r="AJ10" s="1"/>
+      <c r="AK10" s="1"/>
+      <c r="AL10" s="1"/>
+      <c r="AM10" s="1"/>
+      <c r="AN10" s="1"/>
+      <c r="AO10" s="1"/>
+      <c r="AP10" s="1"/>
+      <c r="AQ10" s="1"/>
+      <c r="AR10" s="1"/>
+      <c r="AS10" s="1"/>
+      <c r="AT10" s="1"/>
+      <c r="AU10" s="1"/>
+      <c r="AV10" s="1"/>
+      <c r="AW10" s="1"/>
+      <c r="AX10" s="1"/>
+      <c r="AY10" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>